<commit_message>
Use accounting entity table mapping
</commit_message>
<xml_diff>
--- a/output/ap_opening_payment/未匹配清单_应付期初_20260614.xlsx
+++ b/output/ap_opening_payment/未匹配清单_应付期初_20260614.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="206">
   <si>
     <t>未匹配_经办人(工号)</t>
   </si>
@@ -158,6 +158,9 @@
     <t>VSPN GROUP LIMITED</t>
   </si>
   <si>
+    <t>Virtual Sports Co., Ltd</t>
+  </si>
+  <si>
     <t>Virtual Sports Pte. LTD.</t>
   </si>
   <si>
@@ -392,19 +395,19 @@
     <t>王瑶1</t>
   </si>
   <si>
-    <t>17000</t>
-  </si>
-  <si>
-    <t>9000</t>
-  </si>
-  <si>
-    <t>1000</t>
-  </si>
-  <si>
-    <t>3000</t>
-  </si>
-  <si>
-    <t>11000</t>
+    <t>017000</t>
+  </si>
+  <si>
+    <t>009000</t>
+  </si>
+  <si>
+    <t>001000</t>
+  </si>
+  <si>
+    <t>003000</t>
+  </si>
+  <si>
+    <t>011000</t>
   </si>
   <si>
     <t>上海博思智能科技有限公司</t>
@@ -1205,7 +1208,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1231,6 +1234,11 @@
     <row r="5" spans="1:1">
       <c r="A5" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1245,22 +1253,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1275,120 +1283,120 @@
   <sheetData>
     <row r="1" spans="1:24">
       <c r="A1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="O1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Q1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="R1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="S1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="T1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="U1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="V1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="W1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="X1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:24">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="S2">
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X2">
         <v>1420</v>
@@ -1396,46 +1404,46 @@
     </row>
     <row r="3" spans="1:24">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="S3">
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X3">
         <v>1420</v>
@@ -1443,46 +1451,46 @@
     </row>
     <row r="4" spans="1:24">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S4">
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X4">
         <v>1420</v>
@@ -1490,46 +1498,46 @@
     </row>
     <row r="5" spans="1:24">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S5">
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X5">
         <v>1420</v>
@@ -1537,46 +1545,46 @@
     </row>
     <row r="6" spans="1:24">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="S6">
         <v>0</v>
       </c>
       <c r="T6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X6">
         <v>1420</v>
@@ -1584,46 +1592,46 @@
     </row>
     <row r="7" spans="1:24">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="S7">
         <v>0</v>
       </c>
       <c r="T7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U7" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X7">
         <v>1420</v>
@@ -1631,46 +1639,46 @@
     </row>
     <row r="8" spans="1:24">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Q8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S8">
         <v>0</v>
       </c>
       <c r="T8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X8">
         <v>1420</v>
@@ -1678,46 +1686,46 @@
     </row>
     <row r="9" spans="1:24">
       <c r="A9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Q9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S9">
         <v>0</v>
       </c>
       <c r="T9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X9">
         <v>1420</v>
@@ -1725,46 +1733,46 @@
     </row>
     <row r="10" spans="1:24">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="S10">
         <v>0</v>
       </c>
       <c r="T10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X10">
         <v>1420</v>
@@ -1772,46 +1780,46 @@
     </row>
     <row r="11" spans="1:24">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F11" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J11" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="S11">
         <v>0</v>
       </c>
       <c r="T11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="U11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="W11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X11">
         <v>1420</v>
@@ -1819,55 +1827,55 @@
     </row>
     <row r="12" spans="1:24">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L12" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="N12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="O12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="Q12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="S12">
         <v>950</v>
       </c>
       <c r="T12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="U12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="W12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="X12">
         <v>950</v>
@@ -1875,55 +1883,55 @@
     </row>
     <row r="13" spans="1:24">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="N13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="O13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="Q13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="S13">
         <v>950</v>
       </c>
       <c r="T13" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="U13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="W13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="X13">
         <v>950</v>
@@ -1931,58 +1939,58 @@
     </row>
     <row r="14" spans="1:24">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F14" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="L14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="N14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="O14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S14">
         <v>30000</v>
       </c>
       <c r="T14" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="U14" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="W14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X14">
         <v>30000</v>
@@ -1990,58 +1998,58 @@
     </row>
     <row r="15" spans="1:24">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F15" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="L15" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="N15" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="O15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S15">
         <v>30000</v>
       </c>
       <c r="T15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="U15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="W15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X15">
         <v>30000</v>
@@ -2049,49 +2057,49 @@
     </row>
     <row r="16" spans="1:24">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F16" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I16" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J16" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K16" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L16" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="Q16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S16">
         <v>100000</v>
       </c>
       <c r="T16" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U16" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W16" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X16">
         <v>100000</v>
@@ -2099,49 +2107,49 @@
     </row>
     <row r="17" spans="1:24">
       <c r="A17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F17" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I17" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J17" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K17" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L17" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="Q17" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S17">
         <v>100000</v>
       </c>
       <c r="T17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U17" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W17" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X17">
         <v>100000</v>
@@ -2149,49 +2157,49 @@
     </row>
     <row r="18" spans="1:24">
       <c r="A18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K18" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L18" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="Q18" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S18">
         <v>30000</v>
       </c>
       <c r="T18" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W18" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X18">
         <v>30000</v>
@@ -2199,49 +2207,49 @@
     </row>
     <row r="19" spans="1:24">
       <c r="A19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I19" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J19" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K19" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L19" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="Q19" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S19">
         <v>30000</v>
       </c>
       <c r="T19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U19" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W19" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X19">
         <v>30000</v>
@@ -2249,49 +2257,49 @@
     </row>
     <row r="20" spans="1:24">
       <c r="A20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F20" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I20" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K20" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L20" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="Q20" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S20">
         <v>50000</v>
       </c>
       <c r="T20" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U20" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W20" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X20">
         <v>50000</v>
@@ -2299,49 +2307,49 @@
     </row>
     <row r="21" spans="1:24">
       <c r="A21" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C21" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D21" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I21" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J21" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K21" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="Q21" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="S21">
         <v>50000</v>
       </c>
       <c r="T21" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U21" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W21" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X21">
         <v>50000</v>
@@ -2349,58 +2357,58 @@
     </row>
     <row r="22" spans="1:24">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D22" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I22" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="L22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O22" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P22" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="Q22" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="S22">
         <v>5000</v>
       </c>
       <c r="T22" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="U22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="W22" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X22">
         <v>5000</v>
@@ -2408,58 +2416,58 @@
     </row>
     <row r="23" spans="1:24">
       <c r="A23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C23" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D23" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J23" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="L23" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N23" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O23" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P23" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="Q23" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="S23">
         <v>5000</v>
       </c>
       <c r="T23" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="U23" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="W23" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X23">
         <v>5000</v>
@@ -2467,49 +2475,49 @@
     </row>
     <row r="24" spans="1:24">
       <c r="A24" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D24" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E24" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J24" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L24" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q24" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="S24">
         <v>10000</v>
       </c>
       <c r="T24" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U24" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W24" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X24">
         <v>10000</v>
@@ -2517,49 +2525,49 @@
     </row>
     <row r="25" spans="1:24">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C25" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D25" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E25" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J25" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K25" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L25" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q25" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="S25">
         <v>10000</v>
       </c>
       <c r="T25" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U25" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W25" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X25">
         <v>10000</v>
@@ -2567,49 +2575,49 @@
     </row>
     <row r="26" spans="1:24">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D26" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I26" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J26" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K26" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q26" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="S26">
         <v>15000</v>
       </c>
       <c r="T26" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U26" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W26" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X26">
         <v>15000</v>
@@ -2617,49 +2625,49 @@
     </row>
     <row r="27" spans="1:24">
       <c r="A27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D27" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E27" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I27" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J27" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L27" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q27" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="S27">
         <v>15000</v>
       </c>
       <c r="T27" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U27" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W27" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X27">
         <v>15000</v>
@@ -2667,49 +2675,49 @@
     </row>
     <row r="28" spans="1:24">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B28" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C28" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D28" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E28" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J28" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K28" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q28" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="S28">
         <v>20000</v>
       </c>
       <c r="T28" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U28" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W28" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X28">
         <v>20000</v>
@@ -2717,49 +2725,49 @@
     </row>
     <row r="29" spans="1:24">
       <c r="A29" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C29" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F29" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L29" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q29" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="S29">
         <v>20000</v>
       </c>
       <c r="T29" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U29" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W29" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X29">
         <v>20000</v>
@@ -2767,46 +2775,46 @@
     </row>
     <row r="30" spans="1:24">
       <c r="A30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B30" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C30" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D30" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E30" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F30" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K30" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q30" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S30">
         <v>100</v>
       </c>
       <c r="T30" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U30" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W30" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X30">
         <v>100</v>
@@ -2814,46 +2822,46 @@
     </row>
     <row r="31" spans="1:24">
       <c r="A31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B31" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C31" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D31" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E31" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J31" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K31" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q31" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S31">
         <v>100</v>
       </c>
       <c r="T31" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U31" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W31" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X31">
         <v>100</v>
@@ -2861,46 +2869,46 @@
     </row>
     <row r="32" spans="1:24">
       <c r="A32" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B32" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C32" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D32" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E32" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F32" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J32" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K32" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q32" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S32">
         <v>100</v>
       </c>
       <c r="T32" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U32" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W32" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X32">
         <v>100</v>
@@ -2908,46 +2916,46 @@
     </row>
     <row r="33" spans="1:24">
       <c r="A33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B33" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C33" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D33" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E33" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K33" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q33" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S33">
         <v>100</v>
       </c>
       <c r="T33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U33" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X33">
         <v>100</v>
@@ -2955,46 +2963,46 @@
     </row>
     <row r="34" spans="1:24">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B34" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C34" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D34" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E34" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F34" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I34" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K34" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q34" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S34">
         <v>100</v>
       </c>
       <c r="T34" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U34" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W34" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X34">
         <v>100</v>
@@ -3002,46 +3010,46 @@
     </row>
     <row r="35" spans="1:24">
       <c r="A35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B35" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E35" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K35" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q35" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S35">
         <v>100</v>
       </c>
       <c r="T35" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U35" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W35" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X35">
         <v>100</v>
@@ -3049,46 +3057,46 @@
     </row>
     <row r="36" spans="1:24">
       <c r="A36" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B36" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C36" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D36" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E36" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F36" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I36" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K36" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q36" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S36">
         <v>100</v>
       </c>
       <c r="T36" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U36" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W36" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X36">
         <v>100</v>
@@ -3096,46 +3104,46 @@
     </row>
     <row r="37" spans="1:24">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C37" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D37" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E37" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F37" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I37" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K37" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q37" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S37">
         <v>200</v>
       </c>
       <c r="T37" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U37" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W37" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X37">
         <v>200</v>
@@ -3143,46 +3151,46 @@
     </row>
     <row r="38" spans="1:24">
       <c r="A38" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C38" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D38" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E38" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F38" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I38" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K38" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q38" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S38">
         <v>200</v>
       </c>
       <c r="T38" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U38" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W38" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X38">
         <v>200</v>
@@ -3190,46 +3198,46 @@
     </row>
     <row r="39" spans="1:24">
       <c r="A39" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B39" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C39" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D39" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E39" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F39" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I39" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J39" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K39" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q39" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S39">
         <v>200</v>
       </c>
       <c r="T39" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U39" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W39" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X39">
         <v>200</v>
@@ -3237,46 +3245,46 @@
     </row>
     <row r="40" spans="1:24">
       <c r="A40" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B40" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C40" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D40" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E40" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F40" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I40" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J40" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K40" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q40" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S40">
         <v>200</v>
       </c>
       <c r="T40" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U40" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W40" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X40">
         <v>200</v>
@@ -3284,46 +3292,46 @@
     </row>
     <row r="41" spans="1:24">
       <c r="A41" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B41" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D41" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E41" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F41" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I41" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J41" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K41" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q41" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="S41">
         <v>200</v>
       </c>
       <c r="T41" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U41" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W41" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X41">
         <v>200</v>
@@ -3331,49 +3339,49 @@
     </row>
     <row r="42" spans="1:24">
       <c r="A42" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B42" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C42" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D42" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E42" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F42" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I42" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J42" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K42" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="Q42" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="S42">
         <v>500</v>
       </c>
       <c r="T42" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U42" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W42" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X42">
         <v>500</v>
@@ -3381,49 +3389,49 @@
     </row>
     <row r="43" spans="1:24">
       <c r="A43" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B43" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C43" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D43" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F43" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I43" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J43" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L43" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="Q43" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="S43">
         <v>500</v>
       </c>
       <c r="T43" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="U43" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="W43" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X43">
         <v>500</v>
@@ -3431,58 +3439,58 @@
     </row>
     <row r="44" spans="1:24">
       <c r="A44" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B44" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C44" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D44" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E44" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F44" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I44" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J44" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="L44" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N44" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="O44" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P44" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="Q44" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="S44">
         <v>172250</v>
       </c>
       <c r="T44" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="U44" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="W44" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X44">
         <v>172250</v>
@@ -3490,58 +3498,58 @@
     </row>
     <row r="45" spans="1:24">
       <c r="A45" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C45" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D45" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E45" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F45" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I45" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J45" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="L45" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="N45" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="O45" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P45" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="Q45" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="S45">
         <v>172250</v>
       </c>
       <c r="T45" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="U45" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="W45" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X45">
         <v>172250</v>
@@ -3549,58 +3557,58 @@
     </row>
     <row r="46" spans="1:24">
       <c r="A46" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B46" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C46" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D46" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E46" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F46" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I46" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J46" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="L46" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N46" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O46" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="P46" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Q46" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="S46">
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="U46" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="W46" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X46">
         <v>63850</v>
@@ -3608,58 +3616,58 @@
     </row>
     <row r="47" spans="1:24">
       <c r="A47" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B47" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D47" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E47" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F47" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I47" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J47" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K47" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="L47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N47" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O47" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="P47" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Q47" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="S47">
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="U47" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="W47" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X47">
         <v>63850</v>
@@ -3667,58 +3675,58 @@
     </row>
     <row r="48" spans="1:24">
       <c r="A48" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C48" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D48" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E48" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F48" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I48" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J48" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K48" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L48" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N48" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O48" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P48" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q48" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="S48">
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="U48" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="W48" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X48">
         <v>12880</v>
@@ -3726,58 +3734,58 @@
     </row>
     <row r="49" spans="1:24">
       <c r="A49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B49" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C49" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D49" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E49" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F49" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I49" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J49" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K49" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L49" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N49" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O49" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P49" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q49" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="S49">
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="U49" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="W49" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X49">
         <v>12880</v>
@@ -3785,58 +3793,58 @@
     </row>
     <row r="50" spans="1:24">
       <c r="A50" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C50" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D50" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E50" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F50" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I50" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J50" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K50" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="L50" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N50" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O50" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P50" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q50" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S50">
         <v>79500</v>
       </c>
       <c r="T50" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="U50" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="W50" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X50">
         <v>79500</v>
@@ -3844,58 +3852,58 @@
     </row>
     <row r="51" spans="1:24">
       <c r="A51" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B51" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C51" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D51" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E51" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F51" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I51" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J51" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="L51" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N51" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O51" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P51" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q51" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S51">
         <v>79500</v>
       </c>
       <c r="T51" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="U51" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="W51" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X51">
         <v>79500</v>
@@ -3903,58 +3911,58 @@
     </row>
     <row r="52" spans="1:24">
       <c r="A52" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B52" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C52" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D52" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E52" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F52" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I52" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J52" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L52" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="N52" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O52" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P52" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q52" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S52">
         <v>84180</v>
       </c>
       <c r="T52" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="U52" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="W52" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X52">
         <v>84180</v>
@@ -3962,58 +3970,58 @@
     </row>
     <row r="53" spans="1:24">
       <c r="A53" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B53" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C53" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D53" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E53" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F53" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I53" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J53" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="K53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L53" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="N53" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O53" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P53" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q53" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="S53">
         <v>84180</v>
       </c>
       <c r="T53" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="U53" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="W53" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="X53">
         <v>84180</v>

</xml_diff>

<commit_message>
Read employee code from hrmresource
</commit_message>
<xml_diff>
--- a/output/ap_opening_payment/未匹配清单_应付期初_20260614.xlsx
+++ b/output/ap_opening_payment/未匹配清单_应付期初_20260614.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="208">
   <si>
     <t>未匹配_经办人(工号)</t>
   </si>
@@ -26,6 +26,12 @@
     <t>保琳</t>
   </si>
   <si>
+    <t>李雪松</t>
+  </si>
+  <si>
+    <t>梁木子（法务用印）</t>
+  </si>
+  <si>
     <t>王珊珊1</t>
   </si>
   <si>
@@ -353,25 +359,25 @@
     <t>AP01-1</t>
   </si>
   <si>
-    <t>V85213</t>
-  </si>
-  <si>
-    <t>V83559</t>
-  </si>
-  <si>
-    <t>V80408</t>
-  </si>
-  <si>
-    <t>X80470</t>
-  </si>
-  <si>
-    <t>V84849</t>
-  </si>
-  <si>
-    <t>X84898</t>
-  </si>
-  <si>
-    <t>X85286</t>
+    <t>6949</t>
+  </si>
+  <si>
+    <t>4956</t>
+  </si>
+  <si>
+    <t>314</t>
+  </si>
+  <si>
+    <t>4091</t>
+  </si>
+  <si>
+    <t>6221</t>
+  </si>
+  <si>
+    <t>6275</t>
+  </si>
+  <si>
+    <t>7294</t>
   </si>
   <si>
     <t>陈彦</t>
@@ -978,7 +984,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -999,6 +1005,16 @@
     <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1013,192 +1029,192 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1213,32 +1229,32 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1253,22 +1269,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1283,120 +1299,120 @@
   <sheetData>
     <row r="1" spans="1:24">
       <c r="A1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="M1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="O1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="P1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="R1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="S1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="T1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="U1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="V1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="W1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="X1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:24">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="Q2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="S2">
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X2">
         <v>1420</v>
@@ -1404,46 +1420,46 @@
     </row>
     <row r="3" spans="1:24">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="Q3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="S3">
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X3">
         <v>1420</v>
@@ -1451,46 +1467,46 @@
     </row>
     <row r="4" spans="1:24">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F4" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="Q4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="S4">
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U4" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X4">
         <v>1420</v>
@@ -1498,46 +1514,46 @@
     </row>
     <row r="5" spans="1:24">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="Q5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="S5">
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U5" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X5">
         <v>1420</v>
@@ -1545,46 +1561,46 @@
     </row>
     <row r="6" spans="1:24">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="Q6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="S6">
         <v>0</v>
       </c>
       <c r="T6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X6">
         <v>1420</v>
@@ -1592,46 +1608,46 @@
     </row>
     <row r="7" spans="1:24">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="Q7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="S7">
         <v>0</v>
       </c>
       <c r="T7" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U7" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W7" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X7">
         <v>1420</v>
@@ -1639,46 +1655,46 @@
     </row>
     <row r="8" spans="1:24">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I8" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="Q8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="S8">
         <v>0</v>
       </c>
       <c r="T8" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W8" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X8">
         <v>1420</v>
@@ -1686,46 +1702,46 @@
     </row>
     <row r="9" spans="1:24">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J9" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="Q9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="S9">
         <v>0</v>
       </c>
       <c r="T9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U9" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W9" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X9">
         <v>1420</v>
@@ -1733,46 +1749,46 @@
     </row>
     <row r="10" spans="1:24">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E10" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="Q10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="S10">
         <v>0</v>
       </c>
       <c r="T10" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U10" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X10">
         <v>1420</v>
@@ -1780,46 +1796,46 @@
     </row>
     <row r="11" spans="1:24">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E11" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="J11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="Q11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="S11">
         <v>0</v>
       </c>
       <c r="T11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="U11" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="W11" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X11">
         <v>1420</v>
@@ -1827,55 +1843,55 @@
     </row>
     <row r="12" spans="1:24">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F12" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="N12" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="O12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="P12" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="Q12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="S12">
         <v>950</v>
       </c>
       <c r="T12" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="U12" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="W12" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="X12">
         <v>950</v>
@@ -1883,55 +1899,55 @@
     </row>
     <row r="13" spans="1:24">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F13" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K13" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="N13" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="O13" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="P13" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="Q13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="S13">
         <v>950</v>
       </c>
       <c r="T13" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="U13" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="W13" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="X13">
         <v>950</v>
@@ -1939,58 +1955,58 @@
     </row>
     <row r="14" spans="1:24">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D14" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F14" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="K14" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="L14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="N14" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O14" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="P14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="Q14" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S14">
         <v>30000</v>
       </c>
       <c r="T14" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="U14" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="W14" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X14">
         <v>30000</v>
@@ -1998,58 +2014,58 @@
     </row>
     <row r="15" spans="1:24">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C15" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F15" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I15" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="K15" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="L15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="N15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="P15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="Q15" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S15">
         <v>30000</v>
       </c>
       <c r="T15" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="U15" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="W15" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X15">
         <v>30000</v>
@@ -2057,49 +2073,49 @@
     </row>
     <row r="16" spans="1:24">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C16" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D16" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E16" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F16" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I16" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J16" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K16" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L16" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q16" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="S16">
         <v>100000</v>
       </c>
       <c r="T16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U16" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W16" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X16">
         <v>100000</v>
@@ -2107,49 +2123,49 @@
     </row>
     <row r="17" spans="1:24">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C17" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D17" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E17" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F17" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I17" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J17" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K17" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L17" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q17" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="S17">
         <v>100000</v>
       </c>
       <c r="T17" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U17" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W17" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X17">
         <v>100000</v>
@@ -2157,49 +2173,49 @@
     </row>
     <row r="18" spans="1:24">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B18" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D18" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E18" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F18" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I18" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J18" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K18" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L18" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q18" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="S18">
         <v>30000</v>
       </c>
       <c r="T18" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U18" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W18" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X18">
         <v>30000</v>
@@ -2207,49 +2223,49 @@
     </row>
     <row r="19" spans="1:24">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C19" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D19" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F19" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I19" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J19" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K19" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L19" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q19" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="S19">
         <v>30000</v>
       </c>
       <c r="T19" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U19" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W19" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X19">
         <v>30000</v>
@@ -2257,49 +2273,49 @@
     </row>
     <row r="20" spans="1:24">
       <c r="A20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E20" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F20" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I20" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J20" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K20" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L20" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q20" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="S20">
         <v>50000</v>
       </c>
       <c r="T20" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U20" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W20" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X20">
         <v>50000</v>
@@ -2307,49 +2323,49 @@
     </row>
     <row r="21" spans="1:24">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D21" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E21" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J21" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K21" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q21" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="S21">
         <v>50000</v>
       </c>
       <c r="T21" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U21" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W21" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X21">
         <v>50000</v>
@@ -2357,58 +2373,58 @@
     </row>
     <row r="22" spans="1:24">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C22" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D22" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F22" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I22" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J22" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="K22" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L22" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="N22" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="O22" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="P22" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="Q22" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="S22">
         <v>5000</v>
       </c>
       <c r="T22" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="U22" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="W22" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X22">
         <v>5000</v>
@@ -2416,58 +2432,58 @@
     </row>
     <row r="23" spans="1:24">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B23" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C23" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D23" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E23" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F23" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I23" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J23" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="K23" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L23" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="N23" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="O23" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="P23" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="Q23" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="S23">
         <v>5000</v>
       </c>
       <c r="T23" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="U23" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="W23" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X23">
         <v>5000</v>
@@ -2475,49 +2491,49 @@
     </row>
     <row r="24" spans="1:24">
       <c r="A24" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B24" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C24" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E24" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F24" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J24" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K24" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L24" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="Q24" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="S24">
         <v>10000</v>
       </c>
       <c r="T24" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U24" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W24" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X24">
         <v>10000</v>
@@ -2525,49 +2541,49 @@
     </row>
     <row r="25" spans="1:24">
       <c r="A25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C25" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D25" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F25" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I25" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J25" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K25" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L25" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="Q25" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="S25">
         <v>10000</v>
       </c>
       <c r="T25" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U25" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W25" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X25">
         <v>10000</v>
@@ -2575,49 +2591,49 @@
     </row>
     <row r="26" spans="1:24">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C26" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D26" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E26" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F26" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I26" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J26" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K26" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L26" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="Q26" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="S26">
         <v>15000</v>
       </c>
       <c r="T26" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U26" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W26" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X26">
         <v>15000</v>
@@ -2625,49 +2641,49 @@
     </row>
     <row r="27" spans="1:24">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C27" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E27" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I27" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J27" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K27" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L27" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="Q27" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="S27">
         <v>15000</v>
       </c>
       <c r="T27" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U27" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W27" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X27">
         <v>15000</v>
@@ -2675,49 +2691,49 @@
     </row>
     <row r="28" spans="1:24">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B28" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C28" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D28" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E28" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F28" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I28" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J28" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K28" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L28" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="Q28" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="S28">
         <v>20000</v>
       </c>
       <c r="T28" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U28" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W28" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X28">
         <v>20000</v>
@@ -2725,49 +2741,49 @@
     </row>
     <row r="29" spans="1:24">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B29" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C29" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E29" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F29" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I29" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J29" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K29" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="L29" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="Q29" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="S29">
         <v>20000</v>
       </c>
       <c r="T29" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U29" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W29" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X29">
         <v>20000</v>
@@ -2775,46 +2791,46 @@
     </row>
     <row r="30" spans="1:24">
       <c r="A30" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B30" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C30" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D30" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E30" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F30" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I30" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J30" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K30" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q30" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S30">
         <v>100</v>
       </c>
       <c r="T30" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U30" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W30" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X30">
         <v>100</v>
@@ -2822,46 +2838,46 @@
     </row>
     <row r="31" spans="1:24">
       <c r="A31" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B31" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C31" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D31" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E31" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I31" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J31" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K31" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q31" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S31">
         <v>100</v>
       </c>
       <c r="T31" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U31" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W31" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X31">
         <v>100</v>
@@ -2869,46 +2885,46 @@
     </row>
     <row r="32" spans="1:24">
       <c r="A32" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B32" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C32" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D32" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F32" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I32" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J32" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K32" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q32" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S32">
         <v>100</v>
       </c>
       <c r="T32" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U32" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W32" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X32">
         <v>100</v>
@@ -2916,46 +2932,46 @@
     </row>
     <row r="33" spans="1:24">
       <c r="A33" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B33" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C33" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D33" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E33" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F33" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K33" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q33" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S33">
         <v>100</v>
       </c>
       <c r="T33" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U33" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W33" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X33">
         <v>100</v>
@@ -2963,46 +2979,46 @@
     </row>
     <row r="34" spans="1:24">
       <c r="A34" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B34" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C34" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D34" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E34" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F34" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I34" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J34" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K34" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q34" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S34">
         <v>100</v>
       </c>
       <c r="T34" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U34" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W34" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X34">
         <v>100</v>
@@ -3010,46 +3026,46 @@
     </row>
     <row r="35" spans="1:24">
       <c r="A35" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B35" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C35" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D35" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E35" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F35" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I35" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J35" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K35" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q35" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S35">
         <v>100</v>
       </c>
       <c r="T35" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U35" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W35" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X35">
         <v>100</v>
@@ -3057,46 +3073,46 @@
     </row>
     <row r="36" spans="1:24">
       <c r="A36" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B36" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C36" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D36" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E36" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F36" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I36" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J36" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K36" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q36" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S36">
         <v>100</v>
       </c>
       <c r="T36" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U36" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W36" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X36">
         <v>100</v>
@@ -3104,46 +3120,46 @@
     </row>
     <row r="37" spans="1:24">
       <c r="A37" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C37" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D37" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E37" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F37" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I37" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J37" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K37" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q37" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S37">
         <v>200</v>
       </c>
       <c r="T37" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U37" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W37" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X37">
         <v>200</v>
@@ -3151,46 +3167,46 @@
     </row>
     <row r="38" spans="1:24">
       <c r="A38" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C38" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D38" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E38" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F38" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I38" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J38" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K38" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q38" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S38">
         <v>200</v>
       </c>
       <c r="T38" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U38" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W38" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X38">
         <v>200</v>
@@ -3198,46 +3214,46 @@
     </row>
     <row r="39" spans="1:24">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B39" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C39" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D39" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E39" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F39" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I39" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J39" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K39" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q39" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S39">
         <v>200</v>
       </c>
       <c r="T39" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U39" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W39" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X39">
         <v>200</v>
@@ -3245,46 +3261,46 @@
     </row>
     <row r="40" spans="1:24">
       <c r="A40" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B40" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C40" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D40" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E40" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F40" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I40" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J40" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K40" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q40" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S40">
         <v>200</v>
       </c>
       <c r="T40" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U40" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W40" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X40">
         <v>200</v>
@@ -3292,46 +3308,46 @@
     </row>
     <row r="41" spans="1:24">
       <c r="A41" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B41" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C41" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D41" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E41" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F41" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I41" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J41" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K41" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="Q41" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="S41">
         <v>200</v>
       </c>
       <c r="T41" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U41" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W41" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X41">
         <v>200</v>
@@ -3339,49 +3355,49 @@
     </row>
     <row r="42" spans="1:24">
       <c r="A42" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B42" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C42" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D42" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E42" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F42" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I42" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J42" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K42" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L42" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="Q42" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="S42">
         <v>500</v>
       </c>
       <c r="T42" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U42" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W42" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X42">
         <v>500</v>
@@ -3389,49 +3405,49 @@
     </row>
     <row r="43" spans="1:24">
       <c r="A43" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B43" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C43" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D43" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E43" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F43" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I43" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J43" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K43" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L43" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="Q43" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="S43">
         <v>500</v>
       </c>
       <c r="T43" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="U43" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W43" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X43">
         <v>500</v>
@@ -3439,58 +3455,58 @@
     </row>
     <row r="44" spans="1:24">
       <c r="A44" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B44" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C44" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D44" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E44" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F44" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I44" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J44" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K44" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="L44" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="N44" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="O44" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P44" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="Q44" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="S44">
         <v>172250</v>
       </c>
       <c r="T44" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="U44" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="W44" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X44">
         <v>172250</v>
@@ -3498,58 +3514,58 @@
     </row>
     <row r="45" spans="1:24">
       <c r="A45" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B45" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D45" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E45" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F45" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I45" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J45" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K45" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="L45" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="N45" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="O45" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="P45" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="Q45" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="S45">
         <v>172250</v>
       </c>
       <c r="T45" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="U45" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="W45" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X45">
         <v>172250</v>
@@ -3557,58 +3573,58 @@
     </row>
     <row r="46" spans="1:24">
       <c r="A46" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C46" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D46" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E46" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F46" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I46" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J46" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K46" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="L46" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="N46" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="O46" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="P46" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="Q46" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="S46">
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="U46" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="W46" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X46">
         <v>63850</v>
@@ -3616,58 +3632,58 @@
     </row>
     <row r="47" spans="1:24">
       <c r="A47" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B47" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C47" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D47" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E47" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F47" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I47" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J47" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K47" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="L47" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="N47" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="O47" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="P47" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="Q47" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="S47">
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="U47" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="W47" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X47">
         <v>63850</v>
@@ -3675,58 +3691,58 @@
     </row>
     <row r="48" spans="1:24">
       <c r="A48" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B48" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C48" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D48" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E48" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F48" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I48" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J48" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K48" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="L48" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="N48" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="O48" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="P48" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Q48" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="S48">
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="U48" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="W48" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X48">
         <v>12880</v>
@@ -3734,58 +3750,58 @@
     </row>
     <row r="49" spans="1:24">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B49" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C49" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D49" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E49" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F49" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I49" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J49" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K49" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="L49" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="N49" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="O49" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="P49" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Q49" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="S49">
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="U49" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="W49" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X49">
         <v>12880</v>
@@ -3793,58 +3809,58 @@
     </row>
     <row r="50" spans="1:24">
       <c r="A50" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B50" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C50" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D50" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E50" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F50" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I50" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J50" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K50" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="L50" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="N50" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="O50" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="P50" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Q50" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="S50">
         <v>79500</v>
       </c>
       <c r="T50" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="U50" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="W50" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X50">
         <v>79500</v>
@@ -3852,58 +3868,58 @@
     </row>
     <row r="51" spans="1:24">
       <c r="A51" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B51" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C51" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D51" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E51" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F51" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I51" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J51" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="L51" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="N51" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="O51" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="P51" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Q51" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="S51">
         <v>79500</v>
       </c>
       <c r="T51" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="U51" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="W51" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X51">
         <v>79500</v>
@@ -3911,58 +3927,58 @@
     </row>
     <row r="52" spans="1:24">
       <c r="A52" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B52" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C52" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D52" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E52" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F52" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I52" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J52" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L52" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="N52" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="O52" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="P52" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Q52" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="S52">
         <v>84180</v>
       </c>
       <c r="T52" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="U52" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="W52" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X52">
         <v>84180</v>
@@ -3970,58 +3986,58 @@
     </row>
     <row r="53" spans="1:24">
       <c r="A53" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B53" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C53" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D53" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E53" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F53" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I53" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J53" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K53" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L53" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="N53" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="O53" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="P53" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="Q53" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="S53">
         <v>84180</v>
       </c>
       <c r="T53" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="U53" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="W53" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="X53">
         <v>84180</v>

</xml_diff>

<commit_message>
Use job title name for employee code
</commit_message>
<xml_diff>
--- a/output/ap_opening_payment/未匹配清单_应付期初_20260614.xlsx
+++ b/output/ap_opening_payment/未匹配清单_应付期初_20260614.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="206">
   <si>
     <t>未匹配_经办人(工号)</t>
   </si>
@@ -26,12 +26,6 @@
     <t>保琳</t>
   </si>
   <si>
-    <t>李雪松</t>
-  </si>
-  <si>
-    <t>梁木子（法务用印）</t>
-  </si>
-  <si>
     <t>王珊珊1</t>
   </si>
   <si>
@@ -359,25 +353,25 @@
     <t>AP01-1</t>
   </si>
   <si>
-    <t>6949</t>
-  </si>
-  <si>
-    <t>4956</t>
-  </si>
-  <si>
-    <t>314</t>
-  </si>
-  <si>
-    <t>4091</t>
-  </si>
-  <si>
-    <t>6221</t>
-  </si>
-  <si>
-    <t>6275</t>
-  </si>
-  <si>
-    <t>7294</t>
+    <t>V85213</t>
+  </si>
+  <si>
+    <t>V83559</t>
+  </si>
+  <si>
+    <t>V80408</t>
+  </si>
+  <si>
+    <t>X80470</t>
+  </si>
+  <si>
+    <t>V84849</t>
+  </si>
+  <si>
+    <t>X84898</t>
+  </si>
+  <si>
+    <t>X85286</t>
   </si>
   <si>
     <t>陈彦</t>
@@ -984,7 +978,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1005,16 +999,6 @@
     <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1029,192 +1013,192 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1229,32 +1213,32 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1269,22 +1253,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1299,120 +1283,120 @@
   <sheetData>
     <row r="1" spans="1:24">
       <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
         <v>54</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>56</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>57</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>58</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>59</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>60</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>61</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>62</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>63</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>64</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>65</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>66</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>67</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>68</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>69</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
         <v>70</v>
       </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
         <v>71</v>
       </c>
-      <c r="S1" t="s">
+      <c r="U1" t="s">
         <v>72</v>
       </c>
-      <c r="T1" t="s">
+      <c r="V1" t="s">
         <v>73</v>
       </c>
-      <c r="U1" t="s">
+      <c r="W1" t="s">
         <v>74</v>
       </c>
-      <c r="V1" t="s">
+      <c r="X1" t="s">
         <v>75</v>
-      </c>
-      <c r="W1" t="s">
-        <v>76</v>
-      </c>
-      <c r="X1" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:24">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="Q2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="S2">
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X2">
         <v>1420</v>
@@ -1420,46 +1404,46 @@
     </row>
     <row r="3" spans="1:24">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="Q3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="S3">
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X3">
         <v>1420</v>
@@ -1467,46 +1451,46 @@
     </row>
     <row r="4" spans="1:24">
       <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" t="s">
         <v>78</v>
       </c>
-      <c r="B4" t="s">
-        <v>80</v>
-      </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="Q4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="S4">
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U4" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X4">
         <v>1420</v>
@@ -1514,46 +1498,46 @@
     </row>
     <row r="5" spans="1:24">
       <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" t="s">
         <v>78</v>
       </c>
-      <c r="B5" t="s">
-        <v>80</v>
-      </c>
       <c r="C5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="Q5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="S5">
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X5">
         <v>1420</v>
@@ -1561,46 +1545,46 @@
     </row>
     <row r="6" spans="1:24">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="Q6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="S6">
         <v>0</v>
       </c>
       <c r="T6" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W6" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X6">
         <v>1420</v>
@@ -1608,46 +1592,46 @@
     </row>
     <row r="7" spans="1:24">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="Q7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="S7">
         <v>0</v>
       </c>
       <c r="T7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X7">
         <v>1420</v>
@@ -1655,46 +1639,46 @@
     </row>
     <row r="8" spans="1:24">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K8" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="Q8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="S8">
         <v>0</v>
       </c>
       <c r="T8" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X8">
         <v>1420</v>
@@ -1702,46 +1686,46 @@
     </row>
     <row r="9" spans="1:24">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F9" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K9" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="Q9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="S9">
         <v>0</v>
       </c>
       <c r="T9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W9" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X9">
         <v>1420</v>
@@ -1749,46 +1733,46 @@
     </row>
     <row r="10" spans="1:24">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J10" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="Q10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="S10">
         <v>0</v>
       </c>
       <c r="T10" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U10" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X10">
         <v>1420</v>
@@ -1796,46 +1780,46 @@
     </row>
     <row r="11" spans="1:24">
       <c r="A11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E11" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J11" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K11" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="Q11" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="S11">
         <v>0</v>
       </c>
       <c r="T11" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="U11" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="W11" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X11">
         <v>1420</v>
@@ -1843,55 +1827,55 @@
     </row>
     <row r="12" spans="1:24">
       <c r="A12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D12" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" t="s">
         <v>112</v>
       </c>
-      <c r="E12" t="s">
-        <v>114</v>
-      </c>
       <c r="F12" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="K12" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="L12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="N12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="O12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="P12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="Q12" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="S12">
         <v>950</v>
       </c>
       <c r="T12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="U12" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="W12" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="X12">
         <v>950</v>
@@ -1899,55 +1883,55 @@
     </row>
     <row r="13" spans="1:24">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C13" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D13" t="s">
+        <v>110</v>
+      </c>
+      <c r="E13" t="s">
         <v>112</v>
       </c>
-      <c r="E13" t="s">
-        <v>114</v>
-      </c>
       <c r="F13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="K13" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="L13" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="N13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="O13" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="P13" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="Q13" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="S13">
         <v>950</v>
       </c>
       <c r="T13" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="U13" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="W13" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="X13">
         <v>950</v>
@@ -1955,58 +1939,58 @@
     </row>
     <row r="14" spans="1:24">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F14" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J14" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K14" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="L14" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="N14" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="O14" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="P14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="Q14" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S14">
         <v>30000</v>
       </c>
       <c r="T14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="U14" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="W14" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X14">
         <v>30000</v>
@@ -2014,58 +1998,58 @@
     </row>
     <row r="15" spans="1:24">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C15" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D15" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E15" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F15" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I15" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K15" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="L15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="N15" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="O15" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="P15" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="Q15" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S15">
         <v>30000</v>
       </c>
       <c r="T15" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="U15" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="W15" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X15">
         <v>30000</v>
@@ -2073,49 +2057,49 @@
     </row>
     <row r="16" spans="1:24">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E16" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F16" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I16" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J16" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K16" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="Q16" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="S16">
         <v>100000</v>
       </c>
       <c r="T16" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U16" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W16" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X16">
         <v>100000</v>
@@ -2123,49 +2107,49 @@
     </row>
     <row r="17" spans="1:24">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D17" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E17" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F17" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I17" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J17" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K17" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L17" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="Q17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="S17">
         <v>100000</v>
       </c>
       <c r="T17" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U17" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W17" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X17">
         <v>100000</v>
@@ -2173,49 +2157,49 @@
     </row>
     <row r="18" spans="1:24">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C18" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D18" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E18" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F18" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I18" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J18" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K18" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L18" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="Q18" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="S18">
         <v>30000</v>
       </c>
       <c r="T18" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U18" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W18" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X18">
         <v>30000</v>
@@ -2223,49 +2207,49 @@
     </row>
     <row r="19" spans="1:24">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E19" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F19" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I19" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J19" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K19" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L19" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="Q19" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="S19">
         <v>30000</v>
       </c>
       <c r="T19" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U19" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W19" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X19">
         <v>30000</v>
@@ -2273,49 +2257,49 @@
     </row>
     <row r="20" spans="1:24">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B20" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C20" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D20" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F20" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I20" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J20" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L20" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="Q20" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="S20">
         <v>50000</v>
       </c>
       <c r="T20" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U20" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W20" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X20">
         <v>50000</v>
@@ -2323,49 +2307,49 @@
     </row>
     <row r="21" spans="1:24">
       <c r="A21" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E21" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I21" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J21" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K21" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L21" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="Q21" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="S21">
         <v>50000</v>
       </c>
       <c r="T21" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U21" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W21" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X21">
         <v>50000</v>
@@ -2373,58 +2357,58 @@
     </row>
     <row r="22" spans="1:24">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B22" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C22" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D22" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E22" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F22" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I22" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J22" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K22" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L22" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="N22" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="O22" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="P22" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="Q22" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="S22">
         <v>5000</v>
       </c>
       <c r="T22" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="U22" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="W22" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X22">
         <v>5000</v>
@@ -2432,58 +2416,58 @@
     </row>
     <row r="23" spans="1:24">
       <c r="A23" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B23" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C23" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D23" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I23" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J23" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L23" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="N23" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="O23" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="P23" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="Q23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="S23">
         <v>5000</v>
       </c>
       <c r="T23" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="U23" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="W23" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X23">
         <v>5000</v>
@@ -2491,49 +2475,49 @@
     </row>
     <row r="24" spans="1:24">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B24" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D24" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E24" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F24" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I24" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J24" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K24" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L24" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="Q24" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="S24">
         <v>10000</v>
       </c>
       <c r="T24" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U24" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W24" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X24">
         <v>10000</v>
@@ -2541,49 +2525,49 @@
     </row>
     <row r="25" spans="1:24">
       <c r="A25" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D25" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E25" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F25" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I25" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J25" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K25" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L25" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="Q25" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="S25">
         <v>10000</v>
       </c>
       <c r="T25" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U25" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W25" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X25">
         <v>10000</v>
@@ -2591,49 +2575,49 @@
     </row>
     <row r="26" spans="1:24">
       <c r="A26" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B26" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C26" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E26" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F26" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I26" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J26" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K26" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L26" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="Q26" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="S26">
         <v>15000</v>
       </c>
       <c r="T26" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U26" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W26" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X26">
         <v>15000</v>
@@ -2641,49 +2625,49 @@
     </row>
     <row r="27" spans="1:24">
       <c r="A27" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B27" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C27" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D27" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E27" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F27" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I27" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J27" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K27" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L27" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="Q27" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="S27">
         <v>15000</v>
       </c>
       <c r="T27" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U27" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W27" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X27">
         <v>15000</v>
@@ -2691,49 +2675,49 @@
     </row>
     <row r="28" spans="1:24">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C28" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D28" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E28" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F28" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I28" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J28" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K28" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L28" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="Q28" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="S28">
         <v>20000</v>
       </c>
       <c r="T28" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U28" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W28" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X28">
         <v>20000</v>
@@ -2741,49 +2725,49 @@
     </row>
     <row r="29" spans="1:24">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D29" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E29" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F29" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I29" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J29" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K29" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L29" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="Q29" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="S29">
         <v>20000</v>
       </c>
       <c r="T29" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U29" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W29" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X29">
         <v>20000</v>
@@ -2791,46 +2775,46 @@
     </row>
     <row r="30" spans="1:24">
       <c r="A30" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C30" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D30" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E30" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F30" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I30" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J30" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K30" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q30" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S30">
         <v>100</v>
       </c>
       <c r="T30" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U30" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W30" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X30">
         <v>100</v>
@@ -2838,46 +2822,46 @@
     </row>
     <row r="31" spans="1:24">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B31" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C31" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D31" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E31" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F31" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I31" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J31" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K31" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q31" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S31">
         <v>100</v>
       </c>
       <c r="T31" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U31" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W31" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X31">
         <v>100</v>
@@ -2885,46 +2869,46 @@
     </row>
     <row r="32" spans="1:24">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B32" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C32" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D32" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E32" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F32" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I32" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J32" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K32" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q32" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S32">
         <v>100</v>
       </c>
       <c r="T32" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U32" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W32" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X32">
         <v>100</v>
@@ -2932,46 +2916,46 @@
     </row>
     <row r="33" spans="1:24">
       <c r="A33" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C33" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D33" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E33" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F33" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I33" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J33" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K33" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q33" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S33">
         <v>100</v>
       </c>
       <c r="T33" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U33" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W33" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X33">
         <v>100</v>
@@ -2979,46 +2963,46 @@
     </row>
     <row r="34" spans="1:24">
       <c r="A34" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B34" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C34" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D34" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E34" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F34" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I34" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J34" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K34" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q34" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S34">
         <v>100</v>
       </c>
       <c r="T34" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U34" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W34" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X34">
         <v>100</v>
@@ -3026,46 +3010,46 @@
     </row>
     <row r="35" spans="1:24">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B35" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C35" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D35" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E35" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F35" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I35" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J35" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K35" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q35" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S35">
         <v>100</v>
       </c>
       <c r="T35" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U35" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W35" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X35">
         <v>100</v>
@@ -3073,46 +3057,46 @@
     </row>
     <row r="36" spans="1:24">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B36" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C36" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D36" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E36" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F36" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I36" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J36" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K36" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q36" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S36">
         <v>100</v>
       </c>
       <c r="T36" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U36" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W36" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X36">
         <v>100</v>
@@ -3120,46 +3104,46 @@
     </row>
     <row r="37" spans="1:24">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C37" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D37" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E37" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F37" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I37" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J37" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K37" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q37" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S37">
         <v>200</v>
       </c>
       <c r="T37" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U37" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W37" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X37">
         <v>200</v>
@@ -3167,46 +3151,46 @@
     </row>
     <row r="38" spans="1:24">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B38" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C38" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D38" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E38" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F38" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I38" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J38" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K38" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q38" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S38">
         <v>200</v>
       </c>
       <c r="T38" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U38" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W38" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X38">
         <v>200</v>
@@ -3214,46 +3198,46 @@
     </row>
     <row r="39" spans="1:24">
       <c r="A39" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B39" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C39" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D39" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E39" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F39" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I39" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J39" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K39" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q39" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S39">
         <v>200</v>
       </c>
       <c r="T39" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U39" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W39" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X39">
         <v>200</v>
@@ -3261,46 +3245,46 @@
     </row>
     <row r="40" spans="1:24">
       <c r="A40" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B40" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C40" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D40" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E40" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F40" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I40" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J40" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K40" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q40" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S40">
         <v>200</v>
       </c>
       <c r="T40" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U40" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W40" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X40">
         <v>200</v>
@@ -3308,46 +3292,46 @@
     </row>
     <row r="41" spans="1:24">
       <c r="A41" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D41" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E41" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F41" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I41" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J41" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K41" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="Q41" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="S41">
         <v>200</v>
       </c>
       <c r="T41" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U41" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W41" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X41">
         <v>200</v>
@@ -3355,49 +3339,49 @@
     </row>
     <row r="42" spans="1:24">
       <c r="A42" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C42" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D42" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E42" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F42" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I42" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J42" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K42" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="L42" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="Q42" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="S42">
         <v>500</v>
       </c>
       <c r="T42" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U42" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W42" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X42">
         <v>500</v>
@@ -3405,49 +3389,49 @@
     </row>
     <row r="43" spans="1:24">
       <c r="A43" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B43" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C43" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D43" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E43" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F43" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I43" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J43" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K43" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="L43" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="Q43" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="S43">
         <v>500</v>
       </c>
       <c r="T43" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U43" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="W43" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X43">
         <v>500</v>
@@ -3455,58 +3439,58 @@
     </row>
     <row r="44" spans="1:24">
       <c r="A44" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B44" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C44" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D44" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E44" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F44" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I44" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="J44" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K44" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L44" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="N44" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="O44" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="P44" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="Q44" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="S44">
         <v>172250</v>
       </c>
       <c r="T44" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="U44" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="W44" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X44">
         <v>172250</v>
@@ -3514,58 +3498,58 @@
     </row>
     <row r="45" spans="1:24">
       <c r="A45" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C45" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D45" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E45" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F45" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I45" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="J45" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K45" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L45" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="N45" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="O45" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="P45" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="Q45" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="S45">
         <v>172250</v>
       </c>
       <c r="T45" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="U45" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="W45" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X45">
         <v>172250</v>
@@ -3573,58 +3557,58 @@
     </row>
     <row r="46" spans="1:24">
       <c r="A46" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B46" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C46" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D46" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E46" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F46" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I46" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J46" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K46" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="L46" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="N46" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O46" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="P46" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="Q46" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="S46">
         <v>0</v>
       </c>
       <c r="T46" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="U46" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="W46" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X46">
         <v>63850</v>
@@ -3632,58 +3616,58 @@
     </row>
     <row r="47" spans="1:24">
       <c r="A47" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B47" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D47" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E47" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F47" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I47" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J47" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K47" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="L47" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="N47" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="O47" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="P47" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="Q47" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="S47">
         <v>0</v>
       </c>
       <c r="T47" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="U47" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="W47" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X47">
         <v>63850</v>
@@ -3691,58 +3675,58 @@
     </row>
     <row r="48" spans="1:24">
       <c r="A48" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B48" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C48" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D48" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E48" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F48" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I48" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J48" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K48" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L48" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="N48" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="O48" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="P48" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="Q48" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="S48">
         <v>0</v>
       </c>
       <c r="T48" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="U48" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="W48" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X48">
         <v>12880</v>
@@ -3750,58 +3734,58 @@
     </row>
     <row r="49" spans="1:24">
       <c r="A49" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B49" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C49" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D49" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E49" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F49" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I49" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J49" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K49" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L49" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="N49" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="O49" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="P49" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="Q49" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="S49">
         <v>0</v>
       </c>
       <c r="T49" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="U49" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="W49" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X49">
         <v>12880</v>
@@ -3809,58 +3793,58 @@
     </row>
     <row r="50" spans="1:24">
       <c r="A50" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B50" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C50" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D50" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E50" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F50" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I50" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J50" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K50" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="L50" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="N50" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="O50" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="P50" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="Q50" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="S50">
         <v>79500</v>
       </c>
       <c r="T50" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="U50" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="W50" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X50">
         <v>79500</v>
@@ -3868,58 +3852,58 @@
     </row>
     <row r="51" spans="1:24">
       <c r="A51" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B51" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C51" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D51" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E51" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F51" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I51" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J51" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K51" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="L51" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="N51" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="O51" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="P51" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="Q51" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="S51">
         <v>79500</v>
       </c>
       <c r="T51" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="U51" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="W51" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X51">
         <v>79500</v>
@@ -3927,58 +3911,58 @@
     </row>
     <row r="52" spans="1:24">
       <c r="A52" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B52" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C52" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D52" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E52" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F52" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I52" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J52" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K52" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="L52" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="N52" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="O52" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="P52" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="Q52" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="S52">
         <v>84180</v>
       </c>
       <c r="T52" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="U52" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="W52" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X52">
         <v>84180</v>
@@ -3986,58 +3970,58 @@
     </row>
     <row r="53" spans="1:24">
       <c r="A53" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B53" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C53" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D53" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E53" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F53" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I53" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J53" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K53" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="L53" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="N53" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="O53" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="P53" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="Q53" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="S53">
         <v>84180</v>
       </c>
       <c r="T53" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="U53" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="W53" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="X53">
         <v>84180</v>

</xml_diff>